<commit_message>
Data Table formatted for clear view
</commit_message>
<xml_diff>
--- a/Day 6/Goal Seek Assignment.xlsx
+++ b/Day 6/Goal Seek Assignment.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{36886872-D4FD-46BD-A981-BF1C3A531210}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{933666C4-595C-489F-AB1E-CEC786006D6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4284" yWindow="3540" windowWidth="17280" windowHeight="9420" xr2:uid="{F5430803-45EC-49E2-9656-254BFE10ACCD}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{F5430803-45EC-49E2-9656-254BFE10ACCD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Item</t>
   </si>
@@ -60,15 +60,23 @@
   <si>
     <t>Profit</t>
   </si>
-  <si>
-    <t>?</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+  </numFmts>
+  <fonts count="4" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -78,7 +86,14 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -93,7 +108,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -101,32 +116,236 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="6">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -137,6 +356,17 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BC774AE7-9C8E-4184-B9B7-63EBAD6F01A5}" name="Table1" displayName="Table1" ref="A1:B7" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="4" tableBorderDxfId="5" totalsRowBorderDxfId="3">
+  <autoFilter ref="A1:B7" xr:uid="{BC774AE7-9C8E-4184-B9B7-63EBAD6F01A5}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{744F0AFD-BE83-43B0-BC0F-8A5A3906C2F1}" name="Item" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{123A748C-32FA-404F-A44C-F8D01AE9D0B4}" name="Value" dataDxfId="0" dataCellStyle="Comma"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -439,66 +669,72 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="13.21875" customWidth="1"/>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="21.33203125" customWidth="1"/>
+    <col min="3" max="3" width="41.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:2" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:2" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="6">
         <v>200000</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
+    <row r="3" spans="1:2" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="6">
         <v>100000</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+    <row r="4" spans="1:2" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="6">
         <v>50000</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
+    <row r="5" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="7">
         <v>350000</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
+    <row r="6" spans="1:2" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="6">
         <v>5000</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
+    <row r="7" spans="1:2" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>8</v>
+      <c r="B7" s="8">
+        <v>500000</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem Set and Profit formula is applied
</commit_message>
<xml_diff>
--- a/Day 6/Goal Seek Assignment.xlsx
+++ b/Day 6/Goal Seek Assignment.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{933666C4-595C-489F-AB1E-CEC786006D6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{448DD32B-8E97-457E-8DAD-0AF7204F72F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{F5430803-45EC-49E2-9656-254BFE10ACCD}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="11">
   <si>
     <t>Item</t>
   </si>
@@ -58,7 +58,16 @@
     <t>Course Fee</t>
   </si>
   <si>
-    <t>Profit</t>
+    <t>Student</t>
+  </si>
+  <si>
+    <t>Problem: A school has 100 students, how much course fee should be set to make 500000tk profit?</t>
+  </si>
+  <si>
+    <t>Students</t>
+  </si>
+  <si>
+    <t>Profit Target</t>
   </si>
 </sst>
 </file>
@@ -69,7 +78,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -79,6 +88,20 @@
     </font>
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -99,13 +122,37 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="16"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor theme="0" tint="-0.14999847407452621"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="7">
@@ -187,38 +234,49 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Accent4" xfId="2" builtinId="41"/>
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -666,15 +724,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B8CF19E-DB3A-4457-92A3-A496816E854F}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="2" width="21.33203125" customWidth="1"/>
-    <col min="3" max="3" width="41.77734375" customWidth="1"/>
+    <col min="3" max="3" width="16.21875" customWidth="1"/>
+    <col min="4" max="4" width="25.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -682,7 +741,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -690,7 +749,7 @@
         <v>200000</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
@@ -698,7 +757,7 @@
         <v>100000</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
@@ -706,7 +765,7 @@
         <v>50000</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
@@ -714,20 +773,55 @@
         <v>350000</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B6" s="6">
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B7" s="8">
         <v>500000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+      <c r="A9" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="11"/>
+    </row>
+    <row r="11" spans="1:4" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="21" x14ac:dyDescent="0.3">
+      <c r="A12" s="12">
+        <v>100</v>
+      </c>
+      <c r="B12" s="12"/>
+      <c r="C12" s="12">
+        <v>350000</v>
+      </c>
+      <c r="D12" s="12">
+        <f>(A12*B12)-C12</f>
+        <v>-350000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
What if Goal Seek Analysis is done
</commit_message>
<xml_diff>
--- a/Day 6/Goal Seek Assignment.xlsx
+++ b/Day 6/Goal Seek Assignment.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{448DD32B-8E97-457E-8DAD-0AF7204F72F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EC0AE03-7015-438F-9D16-FE215ED7C959}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{F5430803-45EC-49E2-9656-254BFE10ACCD}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="12">
   <si>
     <t>Item</t>
   </si>
@@ -68,6 +68,9 @@
   </si>
   <si>
     <t>Profit Target</t>
+  </si>
+  <si>
+    <t>After What if Goal Seek Analysis we have found Course Fee should be 8500tk to make 500000tk Profit.</t>
   </si>
 </sst>
 </file>
@@ -130,7 +133,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -139,7 +142,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7"/>
+        <fgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
       </patternFill>
     </fill>
     <fill>
@@ -155,7 +163,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -164,6 +172,21 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right style="thin">
         <color indexed="64"/>
@@ -237,46 +260,50 @@
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Accent4" xfId="2" builtinId="41"/>
+    <cellStyle name="Accent6" xfId="2" builtinId="49"/>
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -724,7 +751,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B8CF19E-DB3A-4457-92A3-A496816E854F}">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -733,7 +760,7 @@
     <col min="4" max="4" width="25.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -741,7 +768,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -749,7 +776,7 @@
         <v>200000</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
@@ -757,7 +784,7 @@
         <v>100000</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
@@ -765,7 +792,7 @@
         <v>50000</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
@@ -773,7 +800,7 @@
         <v>350000</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>7</v>
       </c>
@@ -781,7 +808,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>10</v>
       </c>
@@ -789,40 +816,56 @@
         <v>500000</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
         <v>8</v>
       </c>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
       <c r="D9" s="11"/>
-    </row>
-    <row r="11" spans="1:4" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="13" t="s">
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+    </row>
+    <row r="11" spans="1:7" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="13" t="s">
+      <c r="B11" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="D11" s="15" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="21" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" ht="21" x14ac:dyDescent="0.3">
       <c r="A12" s="12">
         <v>100</v>
       </c>
-      <c r="B12" s="12"/>
+      <c r="B12" s="13">
+        <v>8500</v>
+      </c>
       <c r="C12" s="12">
         <v>350000</v>
       </c>
       <c r="D12" s="12">
         <f>(A12*B12)-C12</f>
-        <v>-350000</v>
-      </c>
+        <v>500000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="18" x14ac:dyDescent="0.35">
+      <c r="A14" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+      <c r="G14" s="14"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>